<commit_message>
Practitioner.identifier.type obligatoire & ADELI interdit (#249)
* update following discussions

* Update AsPractitionerProfile.fsh

* Update AsPractitionerProfile.fsh

* Update AsDpPractitionerProfile.fsh cda7110388a9a42edbeaaa14fd6c4fa68bfe6177
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-as-dp-practitioner.xlsx
+++ b/main/ig/StructureDefinition-as-dp-practitioner.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-01-31T09:33:18+00:00</t>
+    <t>2025-02-03T16:26:04+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -23709,7 +23709,7 @@
       </c>
       <c r="E150" s="2"/>
       <c r="F150" t="s" s="2">
-        <v>85</v>
+        <v>102</v>
       </c>
       <c r="G150" t="s" s="2">
         <v>102</v>
@@ -24928,7 +24928,7 @@
       </c>
       <c r="E159" s="2"/>
       <c r="F159" t="s" s="2">
-        <v>85</v>
+        <v>102</v>
       </c>
       <c r="G159" t="s" s="2">
         <v>102</v>

</xml_diff>